<commit_message>
update electrolyser load in function (sec -> hours)
</commit_message>
<xml_diff>
--- a/data_ProjectTemplate/Electrolysers_ProjectTemplate.xlsx
+++ b/data_ProjectTemplate/Electrolysers_ProjectTemplate.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AteHe\Desktop\Modellen\Zero_ProjectTemplate\data_ProjectTemplate\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AteHe\Desktop\Modellen\data_Generic\data_ProjectTemplate\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2D14B1D-9067-4666-8E43-0C4C5B3C1367}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{201694D9-0A06-4449-9286-400BC4683EFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="electrolysers" sheetId="2" r:id="rId1"/>
@@ -687,18 +687,6 @@
     <t>latitude</t>
   </si>
   <si>
-    <t>load_change_time_s</t>
-  </si>
-  <si>
-    <t>start_up_time_idle_s</t>
-  </si>
-  <si>
-    <t>start_up_time_standby_s</t>
-  </si>
-  <si>
-    <t>start_up_time_shutdown_s</t>
-  </si>
-  <si>
     <t>idle_consumption_power_ratio</t>
   </si>
   <si>
@@ -754,6 +742,18 @@
   </si>
   <si>
     <t>gridnode_id</t>
+  </si>
+  <si>
+    <t>load_change_time_h</t>
+  </si>
+  <si>
+    <t>start_up_time_idle_h</t>
+  </si>
+  <si>
+    <t>start_up_time_standby_h</t>
+  </si>
+  <si>
+    <t>start_up_time_shutdown_h</t>
   </si>
 </sst>
 </file>
@@ -1136,73 +1136,73 @@
   <sheetData>
     <row r="1" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="O1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="P1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="Q1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="R1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="S1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="T1" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="U1" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="V1" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="W1" s="2" t="s">
         <v>22</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="J1" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="K1" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="L1" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="M1" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="N1" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="O1" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="P1" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="Q1" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="R1" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="S1" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="T1" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="U1" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="V1" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="W1" s="2" t="s">
-        <v>3</v>
       </c>
       <c r="X1" s="2" t="s">
         <v>2</v>

</xml_diff>